<commit_message>
Fix typo in SSMs MG template where it said tomocyntes instead of tomosyntes
</commit_message>
<xml_diff>
--- a/Rapportering/Arsstatistik/ReportTemplates/MAM Mall årsredovisning DosReg 2025.xlsx
+++ b/Rapportering/Arsstatistik/ReportTemplates/MAM Mall årsredovisning DosReg 2025.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10201"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Dosreg\Ändringar i statistik 2024\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/josef/Documents/RVB/Programming/rvbrtg/Rapportering/Arsstatistik/ReportTemplates/"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33CAD020-6C04-5148-BFE1-52B1E9AEDA4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="16980"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="16980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MA" sheetId="3" r:id="rId1"/>
@@ -77,9 +78,6 @@
     <t>MAM2</t>
   </si>
   <si>
-    <t>Bröstkörtlar tomocyntes</t>
-  </si>
-  <si>
     <t>MAM3</t>
   </si>
   <si>
@@ -111,12 +109,15 @@
   </si>
   <si>
     <t>-</t>
+  </si>
+  <si>
+    <t>Bröstkörtlar tomosyntes</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -175,7 +176,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -183,18 +184,16 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -474,51 +473,51 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:P7"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="4" max="4" width="27.90625" customWidth="1"/>
-    <col min="5" max="6" width="14.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="27.83203125" customWidth="1"/>
+    <col min="5" max="6" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.5" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="13" customWidth="1"/>
-    <col min="9" max="9" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="7.08984375" customWidth="1"/>
-    <col min="11" max="11" width="6.08984375" customWidth="1"/>
-    <col min="12" max="12" width="14.08984375" customWidth="1"/>
-    <col min="13" max="13" width="9.7265625" customWidth="1"/>
-    <col min="14" max="14" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="7.08984375" customWidth="1"/>
-    <col min="16" max="16" width="6.08984375" customWidth="1"/>
+    <col min="9" max="9" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="7.1640625" customWidth="1"/>
+    <col min="11" max="11" width="6.1640625" customWidth="1"/>
+    <col min="12" max="12" width="14.1640625" customWidth="1"/>
+    <col min="13" max="13" width="9.6640625" customWidth="1"/>
+    <col min="14" max="14" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="7.1640625" customWidth="1"/>
+    <col min="16" max="16" width="6.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>11</v>
       </c>
       <c r="D1" s="4"/>
-      <c r="E1" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
+      <c r="E1" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
       <c r="H1" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I1" s="9"/>
       <c r="J1" s="9"/>
       <c r="K1" s="10"/>
-      <c r="L1" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="M1" s="6" t="s">
+      <c r="L1" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="N1" s="6"/>
-      <c r="O1" s="6"/>
-      <c r="P1" s="6"/>
+      <c r="M1" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="N1" s="9"/>
+      <c r="O1" s="9"/>
+      <c r="P1" s="9"/>
     </row>
-    <row r="2" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>7</v>
       </c>
@@ -549,11 +548,11 @@
       <c r="J2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="K2" s="7" t="s">
+      <c r="K2" s="5" t="s">
         <v>5</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M2" s="3" t="s">
         <v>6</v>
@@ -568,7 +567,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
@@ -581,9 +580,9 @@
       <c r="D3" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="K3" s="8"/>
+      <c r="K3" s="6"/>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>16</v>
       </c>
@@ -594,13 +593,13 @@
         <v>14</v>
       </c>
       <c r="D4" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="K4" s="6"/>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
         <v>17</v>
-      </c>
-      <c r="K4" s="8"/>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
-        <v>18</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>13</v>
@@ -609,62 +608,62 @@
         <v>14</v>
       </c>
       <c r="D5" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="J5" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="K5" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="M5" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N5" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="O5" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="P5" s="8" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="H5" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="I5" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="J5" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="K5" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="M5" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="N5" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="O5" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="P5" s="12" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A6" s="1" t="s">
-        <v>20</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="K6" s="8"/>
+      <c r="K6" s="6"/>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="K7" s="8"/>
+        <v>28</v>
+      </c>
+      <c r="K7" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>